<commit_message>
Updated restd + docs.
</commit_message>
<xml_diff>
--- a/djinterp/docs/restd/restd_coverage.xlsx
+++ b/djinterp/docs/restd/restd_coverage.xlsx
@@ -37,7 +37,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'&lt;tuple&gt;'!$A$4:$Y$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'&lt;type_traits&gt;'!$A$4:$Y$117</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'&lt;utility&gt;'!$A$4:$Y$47</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Pending Dependencies'!$A$4:$E$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Pending Dependencies'!$A$4:$E$49</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Coverage Failures'!$A$4:$F$353</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'Roadmap'!$A$4:$E$21</definedName>
   </definedNames>
@@ -661,12 +661,12 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Single source of truth: coverage_data.py. Builder: build_workbook_v2.py. Style guide: spreadsheet_style.md.</t>
+          <t>Single source of truth: data/*.json. Builder: build_workbook.py. Style guide: spreadsheet_style.md.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="6" customHeight="1"/>
-    <row r="4">
+    <row r="4" ht="22" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Sheets</t>
@@ -723,7 +723,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Per-symbol coverage of the C++ &lt;compare&gt; header (C++20). Phases C1-C4 (2026-05-17) shipped 13 of 17 catalogued symbols: ordering category classes (C1) back-ported to C++11+ via literal_zero_helper; helper meta-functions common_comparison_category + compare_three_way_result (C2); concepts three_way_comparable / three_way_comparable_with (C3); compare_three_way function object and strong_order/weak_order/partial_order niebloids (C4). Phase C5 deferred — *_fallback synthesising CPOs and the floating-point special case in the _order niebloids.</t>
+          <t>Per-symbol coverage of the C++ &lt;compare&gt; header (C++20). Phases C1-C5 (2026-05-17) shipped all 17 catalogued symbols: ordering category classes (C1) back-ported to C++11+; helper meta-functions (C2); concepts three_way_comparable / three_way_comparable_with as SFINAE traits (C3); compare_three_way + strong_order/weak_order/partial_order niebloids (C4); the three compare_*_order_fallback synthesising CPOs (C5). Phase C6 deferred — FP-only special case in strong_order / weak_order for deterministic total order over NaN bit patterns.</t>
         </is>
       </c>
       <c r="C8" s="5" t="n"/>
@@ -863,7 +863,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Symbols that need other restd modules before they reach full coverage. Auto-derived from the depends_on field in coverage_data.py.</t>
+          <t>Symbols that need other restd modules before they reach full coverage. Auto-derived from the depends_on field in the per-header JSON files.</t>
         </is>
       </c>
       <c r="C18" s="5" t="n"/>
@@ -897,7 +897,7 @@
       <c r="C20" s="5" t="n"/>
       <c r="D20" s="6" t="n"/>
     </row>
-    <row r="22">
+    <row r="22" ht="22" customHeight="1">
       <c r="A22" s="3" t="inlineStr">
         <is>
           <t>Colour key</t>
@@ -1030,7 +1030,7 @@
       </c>
       <c r="D29" s="6" t="n"/>
     </row>
-    <row r="31">
+    <row r="31" ht="22" customHeight="1">
       <c r="A31" s="3" t="inlineStr">
         <is>
           <t>Other column meanings</t>
@@ -13413,7 +13413,7 @@
       </c>
       <c r="Y22" s="4" t="inlineStr">
         <is>
-          <t>C++20 spaceship. NOT yet implemented in restd.</t>
+          <t>Shipped 2026-05-17 in tuple/tuple_compare_three_way.hpp. Lexicographic three-way comparison with return type common_comparison_category_t over all element-wise &lt;=&gt; results. Recursive helper internal::tuple_3way_impl walks indices via if constexpr; the identity is strong_ordering::equal cast to the common result type. Arity-matching enforced via a `requires (sizeof...(_A) == sizeof...(_B))` clause. The standard's synth-three-way fallback (from `&lt;` and `==` for types without &lt;=&gt;) is NOT implemented — element types without operator&lt;=&gt; cause a compile error at the decltype site (back-port simplification).</t>
         </is>
       </c>
     </row>
@@ -30647,7 +30647,7 @@
       </c>
       <c r="Y25" s="13" t="inlineStr">
         <is>
-          <t>C++20 spaceship. Pending restd::compare.</t>
+          <t>Shipped 2026-05-17 in utility/pair_compare_three_way.hpp. Two-step lexicographic three-way comparison written inline (pair has fixed arity 2 — no recursive helper needed). Result type is common_comparison_category_t over the two per-element &lt;=&gt; result types. Each per-element &lt;=&gt; result is static_cast'd to the common type before comparison-vs-0 and return.</t>
         </is>
       </c>
     </row>
@@ -33373,7 +33373,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -33393,7 +33393,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Symbols whose full coverage is blocked on a restd module that has not yet shipped. Auto-derived from the depends_on field in coverage_data.py.</t>
+          <t>Symbols whose full coverage is blocked on a restd module that has not yet shipped. Auto-derived from the depends_on field in the per-header JSON files.</t>
         </is>
       </c>
     </row>
@@ -34459,22 +34459,22 @@
       </c>
       <c r="B43" s="13" t="inlineStr">
         <is>
-          <t>operator&lt;=&gt;</t>
+          <t>tuple(allocator_arg, ...)</t>
         </is>
       </c>
       <c r="C43" s="13" t="inlineStr">
         <is>
-          <t>Comparison</t>
+          <t>Allocator interop</t>
         </is>
       </c>
       <c r="D43" s="13" t="inlineStr">
         <is>
-          <t>three_way_comparable</t>
+          <t>allocator_arg_t, uses_allocator</t>
         </is>
       </c>
       <c r="E43" s="13" t="inlineStr">
         <is>
-          <t>C++20 spaceship. NOT yet implemented in restd.</t>
+          <t>Allocator-extended ctor overloads.</t>
         </is>
       </c>
     </row>
@@ -34486,7 +34486,7 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>tuple(allocator_arg, ...)</t>
+          <t>uses_allocator&lt;tuple,A&gt;</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
@@ -34496,56 +34496,56 @@
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>allocator_arg_t, uses_allocator</t>
+          <t>uses_allocator</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>Allocator-extended ctor overloads.</t>
+          <t>Allocator-aware trait specialisation.</t>
         </is>
       </c>
     </row>
     <row r="45" ht="30" customHeight="1">
       <c r="A45" s="13" t="inlineStr">
         <is>
-          <t>&lt;tuple&gt;</t>
+          <t>&lt;type_traits&gt;</t>
         </is>
       </c>
       <c r="B45" s="13" t="inlineStr">
         <is>
-          <t>uses_allocator&lt;tuple,A&gt;</t>
+          <t>invoke_result</t>
         </is>
       </c>
       <c r="C45" s="13" t="inlineStr">
         <is>
-          <t>Allocator interop</t>
+          <t>Transformations</t>
         </is>
       </c>
       <c r="D45" s="13" t="inlineStr">
         <is>
-          <t>uses_allocator</t>
+          <t>reference_wrapper</t>
         </is>
       </c>
       <c r="E45" s="13" t="inlineStr">
         <is>
-          <t>Allocator-aware trait specialisation.</t>
+          <t>Result type of INVOKE(F, Args...). Internal invoker dispatcher hosts the five INVOKE forms; reference_wrapper handling deferred until restd::reference_wrapper lands.</t>
         </is>
       </c>
     </row>
     <row r="46" ht="30" customHeight="1">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>&lt;type_traits&gt;</t>
+          <t>&lt;utility&gt;</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>invoke_result</t>
+          <t>make_pair</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Transformations</t>
+          <t>Factories</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
@@ -34555,7 +34555,7 @@
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>Result type of INVOKE(F, Args...). Internal invoker dispatcher hosts the five INVOKE forms; reference_wrapper handling deferred until restd::reference_wrapper lands.</t>
+          <t>C++11+ uses perfect forwarding with restd::decay; C++98 uses pass-by-value. reference_wrapper unwrap pending restd::reference_wrapper.</t>
         </is>
       </c>
     </row>
@@ -34567,22 +34567,22 @@
       </c>
       <c r="B47" s="13" t="inlineStr">
         <is>
-          <t>make_pair</t>
+          <t>piecewise_construct_t</t>
         </is>
       </c>
       <c r="C47" s="13" t="inlineStr">
         <is>
-          <t>Factories</t>
+          <t>Piecewise construction</t>
         </is>
       </c>
       <c r="D47" s="13" t="inlineStr">
         <is>
-          <t>reference_wrapper</t>
+          <t>tuple</t>
         </is>
       </c>
       <c r="E47" s="13" t="inlineStr">
         <is>
-          <t>C++11+ uses perfect forwarding with restd::decay; C++98 uses pass-by-value. reference_wrapper unwrap pending restd::reference_wrapper.</t>
+          <t>Tag type. Pending restd::tuple.</t>
         </is>
       </c>
     </row>
@@ -34594,7 +34594,7 @@
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>piecewise_construct_t</t>
+          <t>piecewise_construct</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
@@ -34609,7 +34609,7 @@
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>Tag type. Pending restd::tuple.</t>
+          <t>Tag constant. Pending restd::tuple.</t>
         </is>
       </c>
     </row>
@@ -34621,81 +34621,27 @@
       </c>
       <c r="B49" s="13" t="inlineStr">
         <is>
-          <t>piecewise_construct</t>
+          <t>move_if_noexcept</t>
         </is>
       </c>
       <c r="C49" s="13" t="inlineStr">
         <is>
-          <t>Piecewise construction</t>
+          <t>Cast utilities</t>
         </is>
       </c>
       <c r="D49" s="13" t="inlineStr">
         <is>
-          <t>tuple</t>
+          <t>is_nothrow_move_constructible, is_copy_constructible</t>
         </is>
       </c>
       <c r="E49" s="13" t="inlineStr">
         <is>
-          <t>Tag constant. Pending restd::tuple.</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="30" customHeight="1">
-      <c r="A50" s="4" t="inlineStr">
-        <is>
-          <t>&lt;utility&gt;</t>
-        </is>
-      </c>
-      <c r="B50" s="4" t="inlineStr">
-        <is>
-          <t>operator&lt;=&gt; (pair)</t>
-        </is>
-      </c>
-      <c r="C50" s="4" t="inlineStr">
-        <is>
-          <t>Pair comparisons</t>
-        </is>
-      </c>
-      <c r="D50" s="4" t="inlineStr">
-        <is>
-          <t>three_way_comparable</t>
-        </is>
-      </c>
-      <c r="E50" s="4" t="inlineStr">
-        <is>
-          <t>C++20 spaceship. Pending restd::compare.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="30" customHeight="1">
-      <c r="A51" s="13" t="inlineStr">
-        <is>
-          <t>&lt;utility&gt;</t>
-        </is>
-      </c>
-      <c r="B51" s="13" t="inlineStr">
-        <is>
-          <t>move_if_noexcept</t>
-        </is>
-      </c>
-      <c r="C51" s="13" t="inlineStr">
-        <is>
-          <t>Cast utilities</t>
-        </is>
-      </c>
-      <c r="D51" s="13" t="inlineStr">
-        <is>
-          <t>is_nothrow_move_constructible, is_copy_constructible</t>
-        </is>
-      </c>
-      <c r="E51" s="13" t="inlineStr">
-        <is>
           <t>Casts to const T&amp; if T's move can throw and copy is available, else to T&amp;&amp;.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:E51"/>
+  <autoFilter ref="A4:E49"/>
   <mergeCells count="2">
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A1:E1"/>
@@ -35519,12 +35465,12 @@
       </c>
       <c r="E29" s="14" t="inlineStr">
         <is>
-          <t>NOT IMPLEMENTED</t>
+          <t>C++20</t>
         </is>
       </c>
       <c r="F29" s="13" t="inlineStr">
         <is>
-          <t>Phase C5 — synthesis logic for &lt;=&gt;-less types. Needs `&lt;` and `==` SFINAE-detection plus the priority&lt;N&gt; + ADL machinery.</t>
+          <t>Body requires C++20 operator&lt;=&gt; in the priority&lt;2&gt; path; the synth path itself only needs == and &lt;, but the file is gated as a unit.</t>
         </is>
       </c>
     </row>
@@ -35551,12 +35497,12 @@
       </c>
       <c r="E30" s="15" t="inlineStr">
         <is>
-          <t>NOT IMPLEMENTED</t>
+          <t>C++20</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>Phase C5.</t>
+          <t>Same as compare_strong_order_fallback.</t>
         </is>
       </c>
     </row>
@@ -35583,12 +35529,12 @@
       </c>
       <c r="E31" s="14" t="inlineStr">
         <is>
-          <t>NOT IMPLEMENTED</t>
+          <t>C++20</t>
         </is>
       </c>
       <c r="F31" s="13" t="inlineStr">
         <is>
-          <t>Phase C5.</t>
+          <t>Same as compare_strong_order_fallback.</t>
         </is>
       </c>
     </row>
@@ -42571,14 +42517,10 @@
       </c>
       <c r="E262" s="15" t="inlineStr">
         <is>
-          <t>NOT IMPLEMENTED</t>
-        </is>
-      </c>
-      <c r="F262" s="4" t="inlineStr">
-        <is>
-          <t>Requires the C++20 three_way_comparable concept and &lt;compare&gt; ordering categories. Pending restd::compare.</t>
-        </is>
-      </c>
+          <t>C++20</t>
+        </is>
+      </c>
+      <c r="F262" s="4" t="inlineStr"/>
     </row>
     <row r="263" ht="30" customHeight="1">
       <c r="A263" s="13" t="inlineStr">
@@ -44739,14 +44681,10 @@
       </c>
       <c r="E331" s="14" t="inlineStr">
         <is>
-          <t>NOT IMPLEMENTED</t>
-        </is>
-      </c>
-      <c r="F331" s="13" t="inlineStr">
-        <is>
-          <t>Requires the C++20 three_way_comparable concept and &lt;compare&gt; ordering categories. Pending restd::compare.</t>
-        </is>
-      </c>
+          <t>C++20</t>
+        </is>
+      </c>
+      <c r="F331" s="13" t="inlineStr"/>
     </row>
     <row r="332" ht="30" customHeight="1">
       <c r="A332" s="4" t="inlineStr">
@@ -45647,17 +45585,17 @@
       </c>
       <c r="C13" s="13" t="inlineStr">
         <is>
-          <t>Phase C5 — remaining work after Phases C1-C4 shipped 2026-05-17. C1 delivered the three foundational ordering category classes via the literal_zero_helper trick. C2 delivered common_comparison_category + compare_three_way_result plus aliases. C3 delivered three_way_comparable / three_way_comparable_with as SFINAE traits. C4 delivered compare_three_way + the strong_order / weak_order / partial_order niebloids (priority&lt;N&gt; + ADL-poison-pill pattern matching the ranges:: CPOs). Still to ship: C5 — the compare_strong_order_fallback / compare_weak_order_fallback / compare_partial_order_fallback niebloids (synthesising the appropriate category from `&lt;` and `==` when `&lt;=&gt;` is unavailable), and the floating-point special case in the strong_order / weak_order niebloids (deterministic total order over NaN bit patterns).</t>
+          <t>Phase C6 — the only remaining work after Phases C1-C5 shipped 2026-05-17 (all 17 catalogued symbols delivered). C6 covers the floating-point special case in the strong_order / weak_order niebloids: per [cmp.alg], for `float`, `double`, `long double` inputs the niebloid must produce a deterministic total order even across NaN (treating NaN as ordered relative to all finite values, distinguishing +NaN from -NaN, distinguishing -0 from +0). The standard's algorithm operates on the bit pattern; implementations typically use bit_cast (C++20+) or memcpy. Deferred because the rest of the module is functionally complete without it — FP inputs currently route through path (c) of the niebloid and return their built-in partial_ordering, which fails to convert to strong/weak ordering for NaN (compile or runtime mismatch).</t>
         </is>
       </c>
       <c r="D13" s="13" t="inlineStr">
         <is>
-          <t>Body still requires C++20 operator&lt;=&gt;. The fallback CPOs need explicit `&lt;` and `==` SFINAE-detection plus a synthesis function that mirrors the standard's algorithm.</t>
+          <t>Per-platform IEEE-754 sign-and-bit-pattern manipulation, ideally via restd::bit_cast (not yet shipped) or std::memcpy.</t>
         </is>
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>C++20</t>
+          <t>C++20 (refinement)</t>
         </is>
       </c>
     </row>
@@ -60356,7 +60294,7 @@
       </c>
       <c r="Y19" s="13" t="inlineStr">
         <is>
-          <t>Niebloid synthesising a strong_ordering from `&lt;` and `==` when `&lt;=&gt;` is unavailable. Phase C5 work (renamed from C4).</t>
+          <t>Shipped Phase C5 (2026-05-17). Niebloid using priority&lt;N&gt; + trailing-return-SFINAE pattern. Priority&lt;2&gt; defers to the strong_order niebloid (which itself does ADL + built-in &lt;=&gt; dispatch); Priority&lt;1&gt; synthesises from `t == u` and `t &lt; u` via a nested conditional yielding strong_ordering::equal / ::less / ::greater. The same-type constraint from the standard (decay_t&lt;T&gt; == decay_t&lt;U&gt;) is NOT enforced — back-port simplification. Body gated on C++20.</t>
         </is>
       </c>
     </row>
@@ -60479,7 +60417,7 @@
       </c>
       <c r="Y20" s="4" t="inlineStr">
         <is>
-          <t>Niebloid synthesising a weak_ordering. Phase C5 work.</t>
+          <t>Shipped Phase C5 alongside the strong variant. Same dispatch pattern; synth path returns weak_ordering::equivalent / ::less / ::greater. Body gated on C++20.</t>
         </is>
       </c>
     </row>
@@ -60602,7 +60540,7 @@
       </c>
       <c r="Y21" s="13" t="inlineStr">
         <is>
-          <t>Niebloid synthesising a partial_ordering. Phase C5 work.</t>
+          <t>Shipped Phase C5 alongside the other fallbacks. Synth path is one branch longer than strong/weak: tests both `t &lt; u` AND `u &lt; t` so it can produce partial_ordering::unordered when neither ordering holds. Body gated on C++20.</t>
         </is>
       </c>
     </row>

</xml_diff>